<commit_message>
poynt payment integration phase 3B
</commit_message>
<xml_diff>
--- a/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
+++ b/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\Requirement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{973F0398-F95F-496D-B8BD-C515317055B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB00C50-5C41-4C9C-B127-E90E248B7352}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3649FE5F-4067-43E3-9705-A3C81FD1AFF4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
   <si>
     <t>Description</t>
   </si>
@@ -82,6 +82,30 @@
   </si>
   <si>
     <t>Add an approval workflow for the Org admin changes specially Membership/Offers by the owner or specific designated entity.</t>
+  </si>
+  <si>
+    <t>When Customer logs out, URL lands on Org path</t>
+  </si>
+  <si>
+    <t>Sign out is not available easily - not an issue for customers if they are using App But for future reference</t>
+  </si>
+  <si>
+    <t>tax is not calculated when purchased subscription</t>
+  </si>
+  <si>
+    <t>I tried adding staff with duplicate phone number , it didnt give me any error message</t>
+  </si>
+  <si>
+    <t>Staff is saving without name - Critical issue</t>
+  </si>
+  <si>
+    <t>It is working but I think flow is duplicate for saving</t>
+  </si>
+  <si>
+    <t>Not all business shown in the business discovery</t>
+  </si>
+  <si>
+    <t>Membership Edit save is not working</t>
   </si>
 </sst>
 </file>
@@ -515,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7621361-7740-4C28-A3A1-E7CF2DAB5704}">
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -676,6 +700,70 @@
         <v>16</v>
       </c>
     </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
added  poynt cloud api secrets
</commit_message>
<xml_diff>
--- a/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
+++ b/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\Requirement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06EFA235-B238-4FE9-A498-984027721126}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB66937-3996-49E6-8D1A-814508F8376A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3649FE5F-4067-43E3-9705-A3C81FD1AFF4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="39">
   <si>
     <t>Description</t>
   </si>
@@ -106,6 +106,42 @@
   </si>
   <si>
     <t>Membership Edit save is not working</t>
+  </si>
+  <si>
+    <t>Closed</t>
+  </si>
+  <si>
+    <t>No duplicate Business organization onboarding check</t>
+  </si>
+  <si>
+    <t>Add Duplicate Org Admin, Overriding the details if he/she already exists</t>
+  </si>
+  <si>
+    <t>Effective date from and to is timestamp and text field ( should be date field and have calender attached)</t>
+  </si>
+  <si>
+    <t>Country region cities ref data is not being fetched from database</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User and Access screen - no edit button available for new org created by client - available for existing customer only view so not able to set counter operation for org admins. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Benefits -- Multiple product option setting is not working. In the UI multiple products gets selected but when saved it saves only one product id in the DB, it doesn’t show the products on the sumary table on the benfits screen. Interesting when open the benefits in edit mode it still has all the 3 products selected. </t>
+  </si>
+  <si>
+    <t>Products at benefits level is not available foe view by the customer on benefits summary is</t>
+  </si>
+  <si>
+    <t>The same issue with display of multiple products option  mapped to an offer, summary displays all the products linked at th esummary here. Where are the mappings stored?</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Remove/hide indvidual component previews from the screen as it creates confusion with org admin we can renable/view once they are implemented. We can keep just the benefits preview as it is not available until it is added to a membership.</t>
+  </si>
+  <si>
+    <t>Product catalog set up for a new org, the current set up process is not well documented even if it is via DB set up, also add a facility to add these mappings online by upload of excel feature, This is even more important as the org admin is not at all aware of what needs to be done it also involved creation of the integration row which is further down in the set up.</t>
   </si>
 </sst>
 </file>
@@ -230,7 +266,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29FF32A7-DC79-4FBD-B9A8-714797195CD3}" name="Table1" displayName="Table1" ref="A1:E1048576" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{29FF32A7-DC79-4FBD-B9A8-714797195CD3}" name="Table1" displayName="Table1" ref="A1:E1048575" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2" tableBorderDxfId="1">
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{B44FF7F2-6572-4521-B230-947D87E2AF63}" name="Req ID"/>
     <tableColumn id="2" xr3:uid="{D9236474-8678-4CBC-8AEE-26EF86DD1159}" name="Description" dataDxfId="0"/>
@@ -539,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7621361-7740-4C28-A3A1-E7CF2DAB5704}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -572,7 +608,7 @@
         <v>3</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>8</v>
@@ -589,7 +625,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>7</v>
@@ -606,7 +642,7 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>7</v>
@@ -640,7 +676,7 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -657,7 +693,7 @@
         <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
@@ -707,6 +743,9 @@
       <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
+      <c r="C10" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -715,6 +754,9 @@
       <c r="B11" s="5" t="s">
         <v>20</v>
       </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -723,6 +765,9 @@
       <c r="B12" s="5" t="s">
         <v>21</v>
       </c>
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
@@ -731,6 +776,9 @@
       <c r="B13" s="5" t="s">
         <v>22</v>
       </c>
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
@@ -739,6 +787,9 @@
       <c r="B14" s="5" t="s">
         <v>23</v>
       </c>
+      <c r="C14" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
@@ -747,6 +798,9 @@
       <c r="B15" s="5" t="s">
         <v>24</v>
       </c>
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
@@ -755,13 +809,159 @@
       <c r="B16" s="5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" t="s">
+        <v>6</v>
+      </c>
+      <c r="E18" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C19" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" t="s">
+        <v>6</v>
+      </c>
+      <c r="E20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21" t="s">
+        <v>6</v>
+      </c>
+      <c r="E21" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C22" t="s">
+        <v>6</v>
+      </c>
+      <c r="E22" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+      <c r="E23" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C24" t="s">
+        <v>6</v>
+      </c>
+      <c r="E24" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" t="s">
+        <v>6</v>
+      </c>
+      <c r="E25" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" t="s">
+        <v>6</v>
+      </c>
+      <c r="E26" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C27" t="s">
+        <v>6</v>
+      </c>
+      <c r="E27" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Platform Admin add org and business owner
</commit_message>
<xml_diff>
--- a/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
+++ b/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\Requirement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB66937-3996-49E6-8D1A-814508F8376A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE77F2E-515F-48F3-858A-7A277D197BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3649FE5F-4067-43E3-9705-A3C81FD1AFF4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="39">
   <si>
     <t>Description</t>
   </si>
@@ -874,7 +874,7 @@
         <v>31</v>
       </c>
       <c r="C21" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="E21" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Platform Admin Multiple Org admin across org handling
</commit_message>
<xml_diff>
--- a/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
+++ b/docs/Requirement/Requirement_Tracker_Memgine V1.0.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MynikaTech\memgine\docs\Requirement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CE77F2E-515F-48F3-858A-7A277D197BD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D44312-FE2E-47F2-8B26-C766E16D89DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3649FE5F-4067-43E3-9705-A3C81FD1AFF4}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="39">
   <si>
     <t>Description</t>
   </si>
@@ -860,7 +860,7 @@
         <v>30</v>
       </c>
       <c r="C20" t="s">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="E20" t="s">
         <v>36</v>

</xml_diff>